<commit_message>
modify get_unpaired_columns, record SoG, and add main_selisih_lapus.ipynb
</commit_message>
<xml_diff>
--- a/data/output/2025/evaluasi_13.xlsx
+++ b/data/output/2025/evaluasi_13.xlsx
@@ -15,6 +15,14 @@
     <sheet name="1311" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="1309" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="1371" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="1305" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="1307" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="1377" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="1312" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="1373" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="1375" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="1306" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="1376" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -808,6 +816,804 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1307</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kabupaten Agam</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-1.984965940979297</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>q-to-q_pdrb_q4-25_prov vs q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1307</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kabupaten Agam</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20.32982843718013</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1307</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kabupaten Agam</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-1.032974594338031</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>y-on-y_pdrb_q4-25_prov vs y-on-y_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1307</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kabupaten Agam</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.3012257574755403</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>implisit_q-to-q_pdrb_q4-25_prov vs implisit_q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1377</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kota Pariaman</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-1.451067130939746</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>q-to-q_pdrb_q4-25_prov vs q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1377</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kota Pariaman</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2.769905149808413</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1312</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kabupaten Pasaman Barat</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>12.45064742271157</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1312</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kabupaten Pasaman Barat</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2.453765461963487</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1312</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kabupaten Pasaman Barat</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-13.68617966626347</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>y-on-y_pkp_q4-25_prov vs y-on-y_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1373</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kota Sawahlunto</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>29.75756406049726</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1373</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kota Sawahlunto</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.20218221457173</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c-to-c_pmtb_q4-25_prov vs c-to-c_pmtb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1375</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kota Bukittinggi</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.2591111204551158</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>q-to-q_pmtb_q4-25_prov vs q-to-q_pmtb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1375</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kota Bukittinggi</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.7334431841474121</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1375</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kota Bukittinggi</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.8541362926111353</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>implisit_q-to-q_pdrb_q4-25_prov vs implisit_q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1306</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kabupaten Padang Pariaman</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1.932447786871075</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1376</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kota Payakumbuh</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1.018023072914347</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1376</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kota Payakumbuh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-0.6104665899711713</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>implisit_q-to-q_pdrb_q4-25_prov vs implisit_q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -916,7 +1722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1088,6 +1894,90 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Nilai revisi dan nilai rilis beda arah</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1301</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kabupaten Kepulauan Mentawai</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.949562298178605</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>q-to-q_pkrt_q4-25_prov vs q-to-q_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1301</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kabupaten Kepulauan Mentawai</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6.825463936551786</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1301</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kabupaten Kepulauan Mentawai</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2.635438546926724</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1162,6 +2052,118 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Nilai revisi dan nilai rilis beda arah</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1303</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kabupaten Solok</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>14.61424608980625</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1303</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kabupaten Solok</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.3007149283101607</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1303</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kabupaten Solok</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3.490217744503635</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>y-on-y_pmtb_q4-25_prov vs y-on-y_pmtb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1303</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kabupaten Solok</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.1045826123717555</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>c-to-c_pmtb_q4-25_prov vs c-to-c_pmtb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
         </is>
       </c>
     </row>
@@ -1176,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1264,6 +2266,146 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>SoG PI lebih dari +-2 persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1308</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kabupaten Lima Puluh Kota</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-2.771881902934923</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>q-to-q_pdrb_q4-25_prov vs q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kabupaten Lima Puluh Kota</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-1.166132525125275</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>y-on-y_pdrb_q4-25_prov vs y-on-y_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1308</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kabupaten Lima Puluh Kota</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>-28.0771007957145</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>y-on-y_pmtb_q4-25_prov vs y-on-y_pmtb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1308</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kabupaten Lima Puluh Kota</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>-11.05519590477121</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>c-to-c_pmtb_q4-25_prov vs c-to-c_pmtb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1308</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kabupaten Lima Puluh Kota</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>-1.708477067138639</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>implisit_q-to-q_pdrb_q4-25_prov vs implisit_q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
         </is>
       </c>
     </row>
@@ -1278,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1338,6 +2480,90 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Nilai revisi dan nilai rilis beda arah</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1311</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kabupaten Dharmasraya</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>13.07546714037681</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1311</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kabupaten Dharmasraya</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.4347129912864821</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>y-on-y_pkrt_q4-25_prov vs y-on-y_pkrt_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1311</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kabupaten Dharmasraya</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.6189960559213279</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>implisit_q-to-q_pdrb_q4-25_prov vs implisit_q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
         </is>
       </c>
     </row>
@@ -1352,7 +2578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1412,6 +2638,118 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>SoG PI lebih dari +-2 persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1309</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kabupaten Pasaman</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-2.623291189717177</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>q-to-q_pdrb_q4-25_prov vs q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1309</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kabupaten Pasaman</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>17.46113341379607</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1309</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kabupaten Pasaman</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-1.010996508936768</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>y-on-y_pdrb_q4-25_prov vs y-on-y_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1309</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kabupaten Pasaman</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7.100342550247668</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>implisit_y-on-y_pdrb_q4-25_prov vs implisit_y-on-y_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
         </is>
       </c>
     </row>
@@ -1426,7 +2764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1489,6 +2827,248 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1371</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kota Padang</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-0.7652769824402869</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>q-to-q_pdrb_q4-25_prov vs q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1371</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kota Padang</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>17.68818131547545</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kabupaten/kota</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>periode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nilai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kolom</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1305</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kabupaten Tanah Datar</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-2.059293504038135</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>q-to-q_pdrb_q4-25_prov vs q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1305</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kabupaten Tanah Datar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>11.16741861965489</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>q-to-q_pkp_q4-25_prov vs q-to-q_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1305</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kabupaten Tanah Datar</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.5440968726119629</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>y-on-y_pdrb_q4-25_prov vs y-on-y_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1305</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kabupaten Tanah Datar</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-9.134267133224798</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>y-on-y_pkp_q4-25_prov vs y-on-y_pkp_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Selisih dengan nilai provinsi cukup jauh (+-4 point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1305</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kabupaten Tanah Datar</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>q4-25</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>-1.053957610024773</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>implisit_q-to-q_pdrb_q4-25_prov vs implisit_q-to-q_pdrb_q4-25_kab</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Beda arah dengan nilai provinsi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>